<commit_message>
Update In-Transit PO data and Fossil Replenishment page
</commit_message>
<xml_diff>
--- a/data/input/In_Transit_PO data - WM.xlsx
+++ b/data/input/In_Transit_PO data - WM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CFF2CBF-AC9B-41EA-98F9-C75DEF00993C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A95CED4-3EDE-4A96-83CE-D55EA6C1CABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{ED1C42A4-610F-4493-A647-7EDE7899E1B2}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="60">
   <si>
     <t>PO Number</t>
   </si>
@@ -87,9 +87,6 @@
     <t>Delivery Status</t>
   </si>
   <si>
-    <t>Open PO</t>
-  </si>
-  <si>
     <t>ISK3</t>
   </si>
   <si>
@@ -211,6 +208,15 @@
   </si>
   <si>
     <t>WM-HA1M-BK</t>
+  </si>
+  <si>
+    <t>In-Transit</t>
+  </si>
+  <si>
+    <t>5P7LT79E</t>
+  </si>
+  <si>
+    <t>4ZK7TOSG</t>
   </si>
 </sst>
 </file>
@@ -609,7 +615,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD5A3FE4-F9D3-480E-B305-3F537BEA10CA}">
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.296875" bestFit="1" customWidth="1"/>
@@ -682,34 +688,34 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="C2" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D2" s="4">
         <v>46103</v>
       </c>
       <c r="E2" s="4">
-        <v>46112</v>
+        <v>46108</v>
       </c>
       <c r="F2" s="3">
         <v>25269118</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="K2" s="3">
         <v>2</v>
@@ -718,7 +724,7 @@
         <v>2</v>
       </c>
       <c r="M2" s="3">
-        <f t="shared" ref="M2:M10" si="0">K2-L2</f>
+        <f t="shared" ref="M2:M18" si="0">K2-L2</f>
         <v>0</v>
       </c>
       <c r="N2" s="3">
@@ -728,39 +734,39 @@
         <v>4628</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D3" s="4">
         <v>46103</v>
       </c>
       <c r="E3" s="4">
-        <v>46112</v>
+        <v>46108</v>
       </c>
       <c r="F3" s="3">
         <v>25269118</v>
       </c>
       <c r="G3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>28</v>
       </c>
       <c r="K3" s="3">
         <v>1</v>
@@ -779,39 +785,39 @@
         <v>2594</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D4" s="4">
         <v>46103</v>
       </c>
       <c r="E4" s="4">
-        <v>46112</v>
+        <v>46108</v>
       </c>
       <c r="F4" s="3">
         <v>25269118</v>
       </c>
       <c r="G4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>32</v>
       </c>
       <c r="K4" s="3">
         <v>1</v>
@@ -830,39 +836,39 @@
         <v>1721</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D5" s="4">
         <v>46103</v>
       </c>
       <c r="E5" s="4">
-        <v>46112</v>
+        <v>46108</v>
       </c>
       <c r="F5" s="3">
         <v>25269118</v>
       </c>
       <c r="G5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="I5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J5" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>36</v>
       </c>
       <c r="K5" s="3">
         <v>45</v>
@@ -881,39 +887,39 @@
         <v>92700</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D6" s="4">
         <v>46103</v>
       </c>
       <c r="E6" s="4">
-        <v>46112</v>
+        <v>46108</v>
       </c>
       <c r="F6" s="3">
         <v>25269118</v>
       </c>
       <c r="G6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="I6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J6" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>40</v>
       </c>
       <c r="K6" s="3">
         <v>1</v>
@@ -932,39 +938,39 @@
         <v>1297</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D7" s="4">
         <v>46103</v>
       </c>
       <c r="E7" s="4">
-        <v>46112</v>
+        <v>46108</v>
       </c>
       <c r="F7" s="3">
         <v>25269118</v>
       </c>
       <c r="G7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="I7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J7" s="3" t="s">
         <v>43</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>44</v>
       </c>
       <c r="K7" s="3">
         <v>15</v>
@@ -983,39 +989,39 @@
         <v>30510</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D8" s="4">
         <v>46103</v>
       </c>
       <c r="E8" s="4">
-        <v>46112</v>
+        <v>46108</v>
       </c>
       <c r="F8" s="3">
         <v>25269118</v>
       </c>
       <c r="G8" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H8" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="I8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J8" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>48</v>
       </c>
       <c r="K8" s="3">
         <v>5</v>
@@ -1034,39 +1040,39 @@
         <v>15045</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D9" s="4">
         <v>46103</v>
       </c>
       <c r="E9" s="4">
-        <v>46112</v>
+        <v>46108</v>
       </c>
       <c r="F9" s="3">
         <v>25269118</v>
       </c>
       <c r="G9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="H9" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="I9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J9" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>52</v>
       </c>
       <c r="K9" s="3">
         <v>38</v>
@@ -1085,39 +1091,39 @@
         <v>71820</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>54</v>
-      </c>
       <c r="C10" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D10" s="4">
         <v>46104</v>
       </c>
       <c r="E10" s="4">
-        <v>46112</v>
+        <v>46108</v>
       </c>
       <c r="F10" s="3">
         <v>25269117</v>
       </c>
       <c r="G10" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H10" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="I10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J10" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>57</v>
       </c>
       <c r="K10" s="3">
         <v>30</v>
@@ -1136,7 +1142,423 @@
         <v>39150</v>
       </c>
       <c r="P10" s="3" t="s">
-        <v>16</v>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="3" t="str">
+        <f t="shared" ref="B11:B18" si="1">A11&amp;"_"&amp;G11</f>
+        <v>5P7LT79E_B0DP2WC5VW</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="4">
+        <v>46108</v>
+      </c>
+      <c r="E11" s="4">
+        <v>46112</v>
+      </c>
+      <c r="F11" s="3">
+        <v>25269297</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K11" s="3">
+        <v>79</v>
+      </c>
+      <c r="L11" s="3">
+        <v>79</v>
+      </c>
+      <c r="M11" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N11" s="3">
+        <v>2060</v>
+      </c>
+      <c r="O11" s="3">
+        <v>162740</v>
+      </c>
+      <c r="P11" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>5P7LT79E_B0DB5YTQZV</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="4">
+        <v>46108</v>
+      </c>
+      <c r="E12" s="4">
+        <v>46112</v>
+      </c>
+      <c r="F12" s="3">
+        <v>25269297</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="K12" s="3">
+        <v>42</v>
+      </c>
+      <c r="L12" s="3">
+        <v>42</v>
+      </c>
+      <c r="M12" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N12" s="3">
+        <v>2034</v>
+      </c>
+      <c r="O12" s="3">
+        <v>85428</v>
+      </c>
+      <c r="P12" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>5P7LT79E_B0DB5VVPSB</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="4">
+        <v>46108</v>
+      </c>
+      <c r="E13" s="4">
+        <v>46112</v>
+      </c>
+      <c r="F13" s="3">
+        <v>25269297</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="K13" s="3">
+        <v>22</v>
+      </c>
+      <c r="L13" s="3">
+        <v>22</v>
+      </c>
+      <c r="M13" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N13" s="3">
+        <v>3009</v>
+      </c>
+      <c r="O13" s="3">
+        <v>66198</v>
+      </c>
+      <c r="P13" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>5P7LT79E_B0DB5VG39T</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="4">
+        <v>46108</v>
+      </c>
+      <c r="E14" s="4">
+        <v>46112</v>
+      </c>
+      <c r="F14" s="3">
+        <v>25269297</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K14" s="3">
+        <v>81</v>
+      </c>
+      <c r="L14" s="3">
+        <v>81</v>
+      </c>
+      <c r="M14" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N14" s="3">
+        <v>1890</v>
+      </c>
+      <c r="O14" s="3">
+        <v>153090</v>
+      </c>
+      <c r="P14" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>4ZK7TOSG_B0DP32F346</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" s="4">
+        <v>46110</v>
+      </c>
+      <c r="E15" s="4">
+        <v>46112</v>
+      </c>
+      <c r="F15" s="3">
+        <v>25269323</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K15" s="3">
+        <v>1</v>
+      </c>
+      <c r="L15" s="3">
+        <v>1</v>
+      </c>
+      <c r="M15" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N15" s="3">
+        <v>2314</v>
+      </c>
+      <c r="O15" s="3">
+        <v>2314</v>
+      </c>
+      <c r="P15" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>4ZK7TOSG_B0DP2WC5VW</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" s="4">
+        <v>46110</v>
+      </c>
+      <c r="E16" s="4">
+        <v>46112</v>
+      </c>
+      <c r="F16" s="3">
+        <v>25269323</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K16" s="3">
+        <v>1</v>
+      </c>
+      <c r="L16" s="3">
+        <v>1</v>
+      </c>
+      <c r="M16" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N16" s="3">
+        <v>2060</v>
+      </c>
+      <c r="O16" s="3">
+        <v>2060</v>
+      </c>
+      <c r="P16" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>4ZK7TOSG_B0DP2VVRND</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17" s="4">
+        <v>46110</v>
+      </c>
+      <c r="E17" s="4">
+        <v>46112</v>
+      </c>
+      <c r="F17" s="3">
+        <v>25269323</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="K17" s="3">
+        <v>1</v>
+      </c>
+      <c r="L17" s="3">
+        <v>0</v>
+      </c>
+      <c r="M17" s="3">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="N17" s="3">
+        <v>1297</v>
+      </c>
+      <c r="O17" s="3">
+        <v>1297</v>
+      </c>
+      <c r="P17" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>4ZK7TOSG_B0DB5VG39T</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="4">
+        <v>46110</v>
+      </c>
+      <c r="E18" s="4">
+        <v>46112</v>
+      </c>
+      <c r="F18" s="3">
+        <v>25269323</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K18" s="3">
+        <v>1</v>
+      </c>
+      <c r="L18" s="3">
+        <v>1</v>
+      </c>
+      <c r="M18" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N18" s="3">
+        <v>1890</v>
+      </c>
+      <c r="O18" s="3">
+        <v>1890</v>
+      </c>
+      <c r="P18" s="3" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Data: refresh In-Transit PO files (CB + WM)
- In_Transit_PO data.xlsx (CB) — 325 rows
- In_Transit_PO data - WM.xlsx — 9 rows

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/In_Transit_PO data - WM.xlsx
+++ b/data/input/In_Transit_PO data - WM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3C49F85-D50A-4F98-BB7E-93C92D10C44B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1F6490B-75DF-44B4-B10A-7403DE506875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{ED1C42A4-610F-4493-A647-7EDE7899E1B2}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="46">
   <si>
     <t>PO Number</t>
   </si>
@@ -87,9 +87,6 @@
     <t>Delivery Status</t>
   </si>
   <si>
-    <t>4KTSA8KX</t>
-  </si>
-  <si>
     <t>ISK3</t>
   </si>
   <si>
@@ -105,9 +102,6 @@
     <t>HDWF1ML</t>
   </si>
   <si>
-    <t>In-Transit</t>
-  </si>
-  <si>
     <t>B0DP3194QN</t>
   </si>
   <si>
@@ -165,10 +159,22 @@
     <t>WM-GS1M-BK</t>
   </si>
   <si>
-    <t>3UGT4NFD</t>
-  </si>
-  <si>
     <t>Open PO</t>
+  </si>
+  <si>
+    <t>449VTDTK</t>
+  </si>
+  <si>
+    <t>7R9LXN2H</t>
+  </si>
+  <si>
+    <t>B0DP313R77</t>
+  </si>
+  <si>
+    <t>FBA79614</t>
+  </si>
+  <si>
+    <t>MS2ML</t>
   </si>
 </sst>
 </file>
@@ -577,7 +583,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD5A3FE4-F9D3-480E-B305-3F537BEA10CA}">
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.296875" bestFit="1" customWidth="1"/>
@@ -650,359 +656,331 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="B2" s="3" t="str">
         <f>A2&amp;"_"&amp;G2</f>
-        <v>4KTSA8KX_B0DP32F346</v>
+        <v>449VTDTK_B0DP2VVRND</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D2" s="4">
-        <v>46166</v>
-      </c>
-      <c r="E2" s="4">
-        <v>46172</v>
-      </c>
-      <c r="F2" s="3">
-        <v>262701173</v>
-      </c>
+        <v>46176</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="3" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="H2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="I2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>20</v>
-      </c>
       <c r="J2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K2" s="3">
         <v>21</v>
       </c>
-      <c r="K2" s="3">
-        <v>16</v>
-      </c>
       <c r="L2" s="3">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="M2" s="3">
         <v>0</v>
       </c>
       <c r="N2" s="3">
-        <v>2314</v>
+        <v>1297</v>
       </c>
       <c r="O2" s="3">
-        <v>37024</v>
+        <v>27237</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="3" t="str">
+        <f t="shared" ref="B3:B10" si="0">A3&amp;"_"&amp;G3</f>
+        <v>7R9LXN2H_B0DP32F346</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="3" t="str">
-        <f t="shared" ref="B3:B15" si="0">A3&amp;"_"&amp;G3</f>
-        <v>4KTSA8KX_B0DP3194QN</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="4">
+        <v>46180</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="4">
-        <v>46166</v>
-      </c>
-      <c r="E3" s="4">
-        <v>46172</v>
-      </c>
-      <c r="F3" s="3">
-        <v>262701173</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>23</v>
-      </c>
       <c r="H3" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="K3" s="3">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="L3" s="3">
+        <v>49</v>
+      </c>
+      <c r="M3" s="3">
         <v>0</v>
       </c>
-      <c r="M3" s="3">
-        <v>5</v>
-      </c>
       <c r="N3" s="3">
-        <v>2594</v>
+        <v>2314</v>
       </c>
       <c r="O3" s="3">
-        <v>12970</v>
+        <v>113386</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="B4" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>4KTSA8KX_B0DP2WC5VW</v>
+        <v>7R9LXN2H_B0DP3194QN</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D4" s="4">
-        <v>46166</v>
-      </c>
-      <c r="E4" s="4">
-        <v>46172</v>
-      </c>
-      <c r="F4" s="3">
-        <v>262701173</v>
-      </c>
+        <v>46180</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="3"/>
       <c r="G4" s="3" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="K4" s="3">
-        <v>179</v>
+        <v>6</v>
       </c>
       <c r="L4" s="3">
         <v>0</v>
       </c>
       <c r="M4" s="3">
-        <v>179</v>
+        <v>6</v>
       </c>
       <c r="N4" s="3">
-        <v>2060</v>
+        <v>2594</v>
       </c>
       <c r="O4" s="3">
-        <v>368740</v>
+        <v>15564</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="B5" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>4KTSA8KX_B0DP2VVRND</v>
+        <v>7R9LXN2H_B0DP313R77</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D5" s="4">
-        <v>46166</v>
-      </c>
-      <c r="E5" s="4">
-        <v>46172</v>
-      </c>
-      <c r="F5" s="3">
-        <v>262701173</v>
-      </c>
+        <v>46180</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="3"/>
       <c r="G5" s="3" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="K5" s="3">
-        <v>75</v>
+        <v>4</v>
       </c>
       <c r="L5" s="3">
         <v>0</v>
       </c>
       <c r="M5" s="3">
-        <v>75</v>
+        <v>4</v>
       </c>
       <c r="N5" s="3">
-        <v>1297</v>
+        <v>1721</v>
       </c>
       <c r="O5" s="3">
-        <v>97275</v>
+        <v>6884</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="B6" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>4KTSA8KX_B0DB5YTQZV</v>
+        <v>7R9LXN2H_B0DP2WC5VW</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D6" s="4">
-        <v>46166</v>
-      </c>
-      <c r="E6" s="4">
-        <v>46172</v>
-      </c>
-      <c r="F6" s="3">
-        <v>262701173</v>
-      </c>
+        <v>46180</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="3"/>
       <c r="G6" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="K6" s="3">
-        <v>16</v>
+        <v>148</v>
       </c>
       <c r="L6" s="3">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="M6" s="3">
-        <v>0</v>
+        <v>148</v>
       </c>
       <c r="N6" s="3">
-        <v>2034</v>
+        <v>2060</v>
       </c>
       <c r="O6" s="3">
-        <v>32544</v>
+        <v>304880</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="B7" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>4KTSA8KX_B0DB5VVPSB</v>
+        <v>7R9LXN2H_B0DP2VVRND</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D7" s="4">
-        <v>46166</v>
-      </c>
-      <c r="E7" s="4">
-        <v>46172</v>
-      </c>
-      <c r="F7" s="3">
-        <v>262701173</v>
-      </c>
+        <v>46180</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="3"/>
       <c r="G7" s="3" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="K7" s="3">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="L7" s="3">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="M7" s="3">
         <v>0</v>
       </c>
       <c r="N7" s="3">
-        <v>3009</v>
+        <v>1297</v>
       </c>
       <c r="O7" s="3">
-        <v>9027</v>
+        <v>18158</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="B8" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>4KTSA8KX_B0DB5VG39T</v>
+        <v>7R9LXN2H_B0DB5YTQZV</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D8" s="4">
-        <v>46166</v>
-      </c>
-      <c r="E8" s="4">
-        <v>46172</v>
-      </c>
-      <c r="F8" s="3">
-        <v>262701173</v>
-      </c>
+        <v>46180</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="3"/>
       <c r="G8" s="3" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="K8" s="3">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L8" s="3">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M8" s="3">
         <v>0</v>
       </c>
       <c r="N8" s="3">
-        <v>1890</v>
+        <v>2034</v>
       </c>
       <c r="O8" s="3">
-        <v>37800</v>
+        <v>32544</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
@@ -1011,47 +989,45 @@
       </c>
       <c r="B9" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>3UGT4NFD_B0DP32F346</v>
+        <v>7R9LXN2H_B0DB5VVPSB</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D9" s="4">
-        <v>46173</v>
-      </c>
-      <c r="E9" s="4">
-        <v>46179</v>
-      </c>
+        <v>46180</v>
+      </c>
+      <c r="E9" s="4"/>
       <c r="F9" s="3"/>
       <c r="G9" s="3" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="H9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="I9" s="3" t="s">
-        <v>20</v>
-      </c>
       <c r="J9" s="3" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="K9" s="3">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L9" s="3">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M9" s="3">
         <v>0</v>
       </c>
       <c r="N9" s="3">
-        <v>2314</v>
+        <v>3009</v>
       </c>
       <c r="O9" s="3">
-        <v>13884</v>
+        <v>3009</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
@@ -1060,292 +1036,45 @@
       </c>
       <c r="B10" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>3UGT4NFD_B0DP3194QN</v>
+        <v>7R9LXN2H_B0DB5VG39T</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D10" s="4">
-        <v>46173</v>
-      </c>
-      <c r="E10" s="4">
-        <v>46179</v>
-      </c>
+        <v>46180</v>
+      </c>
+      <c r="E10" s="4"/>
       <c r="F10" s="3"/>
       <c r="G10" s="3" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="K10" s="3">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="L10" s="3">
+        <v>28</v>
+      </c>
+      <c r="M10" s="3">
         <v>0</v>
       </c>
-      <c r="M10" s="3">
-        <v>6</v>
-      </c>
       <c r="N10" s="3">
-        <v>2594</v>
+        <v>1890</v>
       </c>
       <c r="O10" s="3">
-        <v>15564</v>
+        <v>52920</v>
       </c>
       <c r="P10" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B11" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>3UGT4NFD_B0DP2WC5VW</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="4">
-        <v>46173</v>
-      </c>
-      <c r="E11" s="4">
-        <v>46179</v>
-      </c>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="K11" s="3">
-        <v>150</v>
-      </c>
-      <c r="L11" s="3">
-        <v>0</v>
-      </c>
-      <c r="M11" s="3">
-        <v>150</v>
-      </c>
-      <c r="N11" s="3">
-        <v>2060</v>
-      </c>
-      <c r="O11" s="3">
-        <v>309000</v>
-      </c>
-      <c r="P11" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B12" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>3UGT4NFD_B0DP2VVRND</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" s="4">
-        <v>46173</v>
-      </c>
-      <c r="E12" s="4">
-        <v>46179</v>
-      </c>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="K12" s="3">
-        <v>58</v>
-      </c>
-      <c r="L12" s="3">
-        <v>0</v>
-      </c>
-      <c r="M12" s="3">
-        <v>58</v>
-      </c>
-      <c r="N12" s="3">
-        <v>1297</v>
-      </c>
-      <c r="O12" s="3">
-        <v>75226</v>
-      </c>
-      <c r="P12" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B13" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>3UGT4NFD_B0DB5YTQZV</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="4">
-        <v>46173</v>
-      </c>
-      <c r="E13" s="4">
-        <v>46179</v>
-      </c>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="K13" s="3">
-        <v>19</v>
-      </c>
-      <c r="L13" s="3">
-        <v>19</v>
-      </c>
-      <c r="M13" s="3">
-        <v>0</v>
-      </c>
-      <c r="N13" s="3">
-        <v>2034</v>
-      </c>
-      <c r="O13" s="3">
-        <v>38646</v>
-      </c>
-      <c r="P13" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B14" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>3UGT4NFD_B0DB5VVPSB</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D14" s="4">
-        <v>46173</v>
-      </c>
-      <c r="E14" s="4">
-        <v>46179</v>
-      </c>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="K14" s="3">
-        <v>1</v>
-      </c>
-      <c r="L14" s="3">
-        <v>1</v>
-      </c>
-      <c r="M14" s="3">
-        <v>0</v>
-      </c>
-      <c r="N14" s="3">
-        <v>3009</v>
-      </c>
-      <c r="O14" s="3">
-        <v>3009</v>
-      </c>
-      <c r="P14" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>3UGT4NFD_B0DB5VG39T</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D15" s="4">
-        <v>46173</v>
-      </c>
-      <c r="E15" s="4">
-        <v>46179</v>
-      </c>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="H15" s="5" t="s">
         <v>40</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="K15" s="3">
-        <v>18</v>
-      </c>
-      <c r="L15" s="3">
-        <v>18</v>
-      </c>
-      <c r="M15" s="3">
-        <v>0</v>
-      </c>
-      <c r="N15" s="3">
-        <v>1890</v>
-      </c>
-      <c r="O15" s="3">
-        <v>34020</v>
-      </c>
-      <c r="P15" s="3" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>